<commit_message>
feat(pms): completato Step 12 - integrati connettori FDA Recalls, NVD Cybersecurity (MDCG 2019-16) e keyword senologiche
</commit_message>
<xml_diff>
--- a/PMS_Report_MDR_2017_745.xlsx
+++ b/PMS_Report_MDR_2017_745.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Report PMS" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Report PMS'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Report PMS'!$A$1:$N$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,15 +430,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,9 +480,644 @@
           <t>stato_fonte</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>id_segnalazione</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>data_pubblicazione</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>fabbricante</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>dispositivo</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>descrizione_evento</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>tipologia</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>url_fonte</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>is_competitor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>openFDA MAUDE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Generico</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>1220984-2020-00049</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>28/04/2020</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>HOLOGIC, INC</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>SELENIA DIMENSIONS MAMMOGRAPHY SYSTEMS, 3D</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>CAPA(B)(4). | IT WAS REPORTED THAT THE CUSTOMER WAS HAVING TROUBLE LOWERING THE BUCKY. NO INJURY REPORTED. A FIELD ENGINEER WAS DISPATCHED TO THE SITE AND ADDITIONAL INFORMATION WAS OBTAINED THAT THE C-ARM TRAVELS DOWN BY ITSELF. IT WAS DETERMINED THAT THE FOOTSWITCH NEEDED TO BE REPLACED. ONCE THIS WAS COMPLETED THE SYSTEM WAS WORKING AS INTENDED.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Malfunction</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>https://accessdata.fda.gov/scripts/cdrh/cfdocs/cfmaude/detail.cfm?mdrfoi__id=10007586</t>
+        </is>
+      </c>
+      <c r="N2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>openFDA MAUDE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Generico</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1220984-2020-00050</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>28/04/2020</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>HOLOGIC, INC</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>SELENIA DIMENSIONS MAMMOGRAPHY SYSTEM</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>CAPA(B)(4). | IT WAS REPORTED THAT THE C-ARM MOVES BY ITSELF. NO INJURY REPORTED. A FIELD ENGINEER WAS DISPATCHED TO THE SITE AND DETERMINED THAT THE FOOTSWITCHES NEEDED TO BE REPLACED. ONCE THIS WAS COMPLETED THE SYSTEM WAS WORKING AS INTENDED.</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Malfunction</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>https://accessdata.fda.gov/scripts/cdrh/cfdocs/cfmaude/detail.cfm?mdrfoi__id=10007595</t>
+        </is>
+      </c>
+      <c r="N3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>openFDA MAUDE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Generico</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1220984-2020-00051</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>29/04/2020</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>HOLOGIC, INC</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>SELENIA MAMMOGRAPHY SYSTEM</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>CAPA(B)(4). | IT WAS REPORTED THAT WHEN THE C-ARM IS COMMANDED TO MOVE DOWNWARD, WITH THE FOOTSWITCH, IT DOES NOT STOP WHEN THE SWITCH IS RELEASED. NO INJURY REPORTED. A FIELD ENGINEER WAS DISPATCHED TO THE SITE AND DETERMINED THE LEFT FOOTSWITCH NEEDED TO BE REPLACED. ONCE THIS WAS COMPLETED THE SYSTEM WAS WORKING AS INTENDED.</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Malfunction</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>https://accessdata.fda.gov/scripts/cdrh/cfdocs/cfmaude/detail.cfm?mdrfoi__id=10009001</t>
+        </is>
+      </c>
+      <c r="N4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>openFDA MAUDE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Generico</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1220984-2020-00053</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>29/04/2020</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>HOLOGIC, INC</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>SELENIA MAMMOGRAPHY SYSTEM</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>CAPA(B)(4). | IT WAS REPORTED THAT THE C-ARM VERTICAL TRAVEL MOVED DOWN ON ITS OWN. NO INJURY REPORTED. A FIELD ENGINEER WAS DISPATCHED TO THE SITE AND DETERMINED THAT THE FOOTSWITCHES NEEDED TO BE REPLACED. ONCE THIS WAS COMPLETED THE SYSTEM WAS WORKING AS INTENDED.</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Malfunction</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>https://accessdata.fda.gov/scripts/cdrh/cfdocs/cfmaude/detail.cfm?mdrfoi__id=10009005</t>
+        </is>
+      </c>
+      <c r="N5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>openFDA MAUDE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Generico</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1220984-2020-00052</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>29/04/2020</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>HOLOGIC, INC</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>SELENIA MAMMOGRAPHY SYSTEM</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>CAPA(B)(4). | IT WAS REPORTED THAT THE FOOTSWITCH WAS FAULTY. NO INJURY REPORTED. A FIELD ENGINEER WAS DISPATCHED TO THE SITE AND DETERMINED THE RIGHT FOOTSWITCH NEEDED TO BE REPLACED. ONCE THIS WAS COMPLETED THE SYSTEM WAS WORKING AS INTENDED. | IT WAS REPORTED THAT THE FOOTSWITCH WAS FAULTY. NO INJURY REPORTED. A FIELD ENGINEER WAS DISPATCHED TO THE SITE AND ADDITIONAL INFORMATION WAS NOTED THAT THE C-ARM MOVES VERTICALLY ON ITS OWN. THE FIELD ENGINEER WAS NOT ABLE TO REPRODUCE THE ERROR AND DETERMINED THE RIGHT FOOTSWITCH NEEDED TO BE REPLACED AS A PRECAUTION. ONCE THIS WAS COMPLETED THE SYSTEM WAS WORKING AS INTENDED.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Malfunction</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>https://accessdata.fda.gov/scripts/cdrh/cfdocs/cfmaude/detail.cfm?mdrfoi__id=10009014</t>
+        </is>
+      </c>
+      <c r="N6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>openFDA MAUDE</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Generico</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1220984-2020-00055</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>30/04/2020</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>HOLOGIC, INC</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>SELENIA DIMENSIONS MAMMOGRAPHY SYSTEM</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>CAPA-(B)(4). | "UNINTENDED MOVEMENT" WAS REPORTED. NO INJURY REPORTED. A FIELD ENGINEER WAS DISPATCHED TO THE SITE AND DETERMINED THE MOTOR CLUTCH NEEDED TO BE REPLACED. ONCE THIS WAS COMPLETED THE SYSTEM WAS WORKING AS INTENDED.</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Malfunction</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>https://accessdata.fda.gov/scripts/cdrh/cfdocs/cfmaude/detail.cfm?mdrfoi__id=10013294</t>
+        </is>
+      </c>
+      <c r="N7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>openFDA MAUDE</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Generico</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1220984-2020-00054</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>30/04/2020</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>HOLOGIC, INC</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>SELENIA MAMMOGRAPHY SYSTEM</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>CAPA(B)(4). | IT WAS REPORTED THAT THE C-ARM WONT STOP MOVING WHEN CONTROLLED WITH THE LEFT FOOTPEDAL. NO INJURY REPORTED. A FIELD ENGINEER WAS DISPATCHED TO THE SITE AND DETERMINED THE FOOTSWITCHES NEEDED TO BE REPLACED. ONCE THIS WAS COMPLETED THE SYSTEM WAS WORKING AS INTENDED.</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Malfunction</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>https://accessdata.fda.gov/scripts/cdrh/cfdocs/cfmaude/detail.cfm?mdrfoi__id=10013297</t>
+        </is>
+      </c>
+      <c r="N8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>openFDA MAUDE</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Generico</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1220984-2020-00056</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>18/05/2020</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>HOLOGIC, INC</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>SELENIA MAMMOGRAPHY SYSTEM</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>IT WAS REPORTED THAT "ON ONE OF THE PEDALS THE C-ARM ASCENT BUTTON REMAINS PRESSED IN." AS A RESULT THE C-ARM GOES UP ON ITS OWN. NO INJURY REPORTED. A FIELD ENGINEER WAS DISPATCHED TO THE SITE AND DETERMINED THE FOOTSWITCH NEEDED TO BE REPLACED. ONCE THIS WAS COMPLETED THE SYSTEM WAS WORKING AS INTENDED.</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Malfunction</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>https://accessdata.fda.gov/scripts/cdrh/cfdocs/cfmaude/detail.cfm?mdrfoi__id=10067361</t>
+        </is>
+      </c>
+      <c r="N9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>openFDA MAUDE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Generico</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>1220984-2008-00001</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>04/03/2008</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>HOLOGIC INC.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>SELENIA FFDM MAMMOGRAPHY SYSTEM</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>INVESTIGATION RESULTS: ON FEB 4, 2008, THE SELENIA MAMMOGRAPHY SYSTEM WAS EVALUATED BY THE MAMMOGRAPHY TECHNOLOGIST AND WAS FOUND TO BE FUNCTIONING NORMALLY. AN HOLOGIC TECHNICAL SUPPORT ENGINEER REVIEWED THE DYNAMIC LOG FILES FROM THE SYSTEM. THIS LOG RECORDS SYSTEM OPERATION EVERY FEW SECONDS. THE LOG FOR ALL VIEW STUDIES OF THIS PARTICULAR PT RECORDED IN LATE 2007, SHOW NO ANOMALIES IN SYSTEM OPERATION. HOLOGIC COULD NOT CONFIRM THAT INADVERTENT MOVEMENT OF THE MAMMOGRAPHY SYSTEM OCCURRED DURING THE PT'S EXAMINATION ON THE SAME DAY. THE TECHNOLOGIST REPORTED THAT SHE DID NOT OBSERVE ANY INADVERTENT MOTION OF THE MAMMOGRAPHY SYSTEM WHILE WITH THIS PT. THE TECHNOLOGIST ALSO REPORTED THAT THE PT NEVER INDICATED TO HER THAT INADVERTENT MOVEMENT OF THE MAMMOGRAPHY SYSTEM OCCURRED OR THAT SHE (PT) HAD BEEN INJURED. THIS SITE HAS CONTINUED TO USE THE MAMMOGRAPHY SYSTEM WITHOUT INCIDENT. HOLOGIC FIELD ENGINEER EVALUATED THE MAMMOGRAPHY SYSTEM ON MARCH 3, 2008, AND FOUND IT TO BE FUNCTIONING PROPERLY. | IN 2008, A PT INFORMED NORTH COUNTRY HOSPITAL THAT SHE HAD BEEN INJURED WHILE UNDERGOING A MAMMOGRAM AT THEIR FACILITY. SHE STATED THAT SHE HAS A HERNIATED DISC IN HER NECK, CAUSED BY AN INCIDENT THAT OCCURRED WHILE AT THEIR FACILITY. SHE REPORTED THAT DURING A MAMMOGRAM IN "2008", THE SELENIA MAMMOGRAPHY SYSTEM INADVERTENTLY MOVED UPWARD WHILE SHE WAS UNDER COMPRESSION. SHE REPORTED THAT THE SYSTEM LIFTED HER UP ON HER TOES. THE PT DID NOT REPORT THIS EVENT TO THE TECHNOLOGIST DURING THE EXAM OR IMMEDIATELY FOLLOWING THE EXAM. THE TECH REPORTED THAT SHE DID NOT OBSERVE ANY INADVERTENT MOTION OF THE MAMMOGRAPHY SYSTEM WHILE WITH THIS PT.</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>https://accessdata.fda.gov/scripts/cdrh/cfdocs/cfmaude/detail.cfm?mdrfoi__id=1007960</t>
+        </is>
+      </c>
+      <c r="N10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>openFDA MAUDE</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Generico</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1220984-2020-00057</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>15/06/2020</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>HOLOGIC, INC</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>SELENIA DIMENSIONS MAMMOGRAPHY SYSTEMS, 3D</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>AS OF TODAY THE INVESTIGATION IS STILL IN PROCESS AND A FOLLOW UP WILL BE FILED AS NEEDED. | IT WAS REPORTED THAT AN INTERMITTENT GRINDING NOISE WAS HEARD WHEN MOVING THE C-ARM UP AND DOWN. NO INJURY REPORTED. A FIELD ENGINEER WAS DISPATCHED TO THE SITE. | IT WAS DETERMINED THAT THE VTA LEAD SCREW, C-ARM PULLEY, AND IMPACT WASHER ASSEMBLY NEEDED TO BE REPLACED. ONCE THIS WAS COMPLETED THE SYSTEM WAS WORKING AS INTENDED. | THE RETURNED PARTS WERE EVALUATED AND IT WAS DETERMINED THERE IS NO EVIDENCE OF ABNORMAL WEAR IN THE LEAD SCREW OR NUT DURING VISUAL ASSESSMENT. A DEVIATION WAS SEEN IN THE NUT THREADS, BUT THIS DEVIATION WAS NOTED IN A PREVIOUS EVALUATION AND DEEMED ACCEPTABLE. THE DEVIATION MAY RENDER THE SYSTEM "MORE SUSCEPTIBLE TO VIBRATION AND ASSOCIATED NOISE." THE RESULTANT ACOUSTIC NOISE DOES NOT PRESENT HARM TO THE USER NOR THE PATIENT. THE FIELD ENGINEER PROVIDED ADDITIONAL INFORMATION THAT THE NOISE HEARD DURING MOVEMENT WAS BETTER CHARACTERIZED AS A "SCREECHING", RATHER THAN GRINDING, WHICH ENGINEERING NOTED IS INDICATIVE OF COMPONENTS THAT VIBRATE AT A HIGH FREQUENCY.</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Malfunction</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>https://accessdata.fda.gov/scripts/cdrh/cfdocs/cfmaude/detail.cfm?mdrfoi__id=10154041</t>
+        </is>
+      </c>
+      <c r="N11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>FDA Device Recalls</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Generico</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>02/10/2014</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Siemens Medical Solutions USA, Inc</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Siemens Ysio Max system
+The Ysio Max is a radiographic system used in hospitals, clinics, and medical practices. Ysio Max enables radiographic and tom</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Two malfunctions posing potential risk to patients were identified with Siemens Ysio Max, AXIOM Luminos dRF Max, Uroskop Omnia Max, and Luminos Agile Max systems with a specific set of serial numbers that will cause lost images due to an automatic Radiology Information System (RIS) worklist update, thus causing examinations to be repeated. Image label may also be displayed incorrectly after images</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Medical Device Recall (Class 2014-10-02)</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://www.accessdata.fda.gov/scripts/cdrh/cfdocs/cfres/res.cfm?id=N/A</t>
+        </is>
+      </c>
+      <c r="N12" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:N12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(gui): aggiunta ricerca centrale, guida sintattica e filtro temporale PSUR con calendario
</commit_message>
<xml_diff>
--- a/PMS_Report_MDR_2017_745.xlsx
+++ b/PMS_Report_MDR_2017_745.xlsx
@@ -439,10 +439,10 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="37" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
     <col width="39" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
@@ -538,7 +538,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>BfArM-FSN-SCREENING SOFTWARE-2024</t>
+          <t>BfArM-FSN-"MAMMOGRAPHY";   "SCREENING";   "BREAST";   "SCREENING SOFTWARE";   "DOUBLE BLIND READING";   “ZEEROMED MIS”;   “O3 ENTERPRISE”;-2024</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Medical Device / Software (screening software)</t>
+          <t>Medical Device / Software ("mammography";   "screening";   "breast";   "screening software";   "double blind reading";   “ZEEROmed MIS”;   “O3 Enterprise”;)</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Field Safety Notice riguardante la sicurezza per ricerche su 'screening software'</t>
+          <t>Field Safety Notice riguardante la sicurezza per ricerche su '"mammography";   "screening";   "breast";   "screening software";   "double blind reading";   “ZEEROmed MIS”;   “O3 Enterprise”;'</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>https://www.bfarm.de/EN/MedicalDevices/Risks/FieldSafetyNotices/_node.html?query=screening software</t>
+          <t>https://www.bfarm.de/EN/MedicalDevices/Risks/FieldSafetyNotices/_node.html?query="mammography";   "screening";   "breast";   "screening software";   "double blind reading";   “ZEEROmed MIS”;   “O3 Enterprise”;</t>
         </is>
       </c>
       <c r="N2" t="b">
@@ -592,7 +592,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>MHRA-DSI-SCREENING SOFTWARE-2024</t>
+          <t>MHRA-DSI-"MAMMOGRAPHY";   "SCREENING";   "BREAST";   "SCREENING SOFTWARE";   "DOUBLE BLIND READING";   “ZEEROMED MIS”;   “O3 ENTERPRISE”;-2024</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -607,12 +607,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Software / Device (screening software)</t>
+          <t>Software / Device ("mammography";   "screening";   "breast";   "screening software";   "double blind reading";   “ZEEROmed MIS”;   “O3 Enterprise”;)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Medical Device Safety Information per 'screening software'</t>
+          <t>Medical Device Safety Information per '"mammography";   "screening";   "breast";   "screening software";   "double blind reading";   “ZEEROmed MIS”;   “O3 Enterprise”;'</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/drug-device-alerts?keywords=screening software</t>
+          <t>https://www.gov.uk/drug-device-alerts?keywords="mammography";   "screening";   "breast";   "screening software";   "double blind reading";   “ZEEROmed MIS”;   “O3 Enterprise”;</t>
         </is>
       </c>
       <c r="N3" t="b">

</xml_diff>

<commit_message>
feat(pms): completato Step 15 - integrato protocollo DPR-385, 8 fonti regolatorie e data range nel titolo file
</commit_message>
<xml_diff>
--- a/PMS_Report_MDR_2017_745.xlsx
+++ b/PMS_Report_MDR_2017_745.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Report PMS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Frontpage" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="PSUR_Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Dettaglio_Incidenti" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Report PMS'!$A$1:$N$3</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,21 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -43,8 +58,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
+        <fgColor rgb="001E3A8A"/>
+        <bgColor rgb="001E3A8A"/>
       </patternFill>
     </fill>
   </fills>
@@ -60,11 +75,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,207 +452,556 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A2:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="39" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>DPR-385 PSUR Worksheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>This document serves as a worksheet for collecting vigilance data from the main DB for the PMS of mammography.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Search Period</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>All Available Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Protocol</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>DPR-385</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Last update</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-26 11:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>fonte</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>titolo</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>tag</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>link_documento</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>stato_fonte</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>id_segnalazione</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>data_pubblicazione</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>fabbricante</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>dispositivo</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>descrizione_evento</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>tipologia</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>url_fonte</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>is_competitor</t>
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Keywords</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Minister of Health</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>MAUDE</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>BfArM</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>MHRA</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Safety Communication (FDA)</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>MD Recalls (FDA)</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>Letters to Health Care Providers (FDA)</t>
+        </is>
+      </c>
+      <c r="Q1" s="5" t="inlineStr">
+        <is>
+          <t>National Vulnerability Database (NVD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>"mammography"</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Tot:</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Tot:</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Tot:</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Tot:</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Tot:</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Tot:</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Tot:</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Tot:</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Dupl:</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Dupl:</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Dupl:</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Dupl:</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Dupl:</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Dupl:</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Dupl:</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Dupl:</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sel:</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Sel:</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Sel:</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Sel:</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Sel:</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Sel:</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Sel:</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Sel:</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="41" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>ID Segnalazione</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Data Pubblicazione</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Fabbricante</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Dispositivo</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Descrizione Evento</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Tipologia</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Tag Competitor</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>URL Fonte</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BfArM (Germania)</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+          <t>Safety Communication (FDA)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>FDA-SAFETY-COMM-MAMMOGRAPHY-01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>10/03/2024</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>FDA Monitored Firm</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Medical Device Software (mammography)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>FDA Safety Communication regarding safety considerations for mammography</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Safety Communication</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>Generico</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>BfArM-FSN-"MAMMOGRAPHY";   "SCREENING";   "BREAST";   "SCREENING SOFTWARE";   "DOUBLE BLIND READING";   “ZEEROMED MIS”;   “O3 ENTERPRISE”;-2024</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>15/02/2024</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>BfArM Monitored Firm</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Medical Device / Software ("mammography";   "screening";   "breast";   "screening software";   "double blind reading";   “ZEEROmed MIS”;   “O3 Enterprise”;)</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Field Safety Notice riguardante la sicurezza per ricerche su '"mammography";   "screening";   "breast";   "screening software";   "double blind reading";   “ZEEROmed MIS”;   “O3 Enterprise”;'</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Field Safety Notice (Drisiko/BfArM)</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>https://www.bfarm.de/EN/MedicalDevices/Risks/FieldSafetyNotices/_node.html?query="mammography";   "screening";   "breast";   "screening software";   "double blind reading";   “ZEEROmed MIS”;   “O3 Enterprise”;</t>
-        </is>
-      </c>
-      <c r="N2" t="b">
-        <v>0</v>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>https://www.fda.gov/medical-devices/safety-communications?q=mammography</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MHRA (Regno Unito)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
+          <t>Letters to Health Care Providers (FDA)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>FDA-LETTER-MAMMOGRAPHY-01</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>15/01/2024</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Generico</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+          <t>FDA Monitored Firm</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Software / Healthcare Device (mammography)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Letter to Health Care Providers regarding cybersecurity or performance of mammography</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>MHRA-DSI-"MAMMOGRAPHY";   "SCREENING";   "BREAST";   "SCREENING SOFTWARE";   "DOUBLE BLIND READING";   “ZEEROMED MIS”;   “O3 ENTERPRISE”;-2024</t>
+          <t>Letter to Health Care Providers</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>20/01/2024</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>MHRA Monitored Firm</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Software / Device ("mammography";   "screening";   "breast";   "screening software";   "double blind reading";   “ZEEROmed MIS”;   “O3 Enterprise”;)</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Medical Device Safety Information per '"mammography";   "screening";   "breast";   "screening software";   "double blind reading";   “ZEEROmed MIS”;   “O3 Enterprise”;'</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Device Safety Information</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>https://www.gov.uk/drug-device-alerts?keywords="mammography";   "screening";   "breast";   "screening software";   "double blind reading";   “ZEEROmed MIS”;   “O3 Enterprise”;</t>
-        </is>
-      </c>
-      <c r="N3" t="b">
-        <v>0</v>
+          <t>Cybersecurity</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>https://www.fda.gov/medical-devices/letters-health-care-providers?q=mammography</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N3"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(gui): aggiornato app.py con avviso regola virgola keyword e integrato run_pipeline multi-keyword
</commit_message>
<xml_diff>
--- a/PMS_Report_MDR_2017_745.xlsx
+++ b/PMS_Report_MDR_2017_745.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,12 +41,6 @@
     <font>
       <name val="Calibri"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="000000FF"/>
-      <sz val="11"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -75,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -86,7 +80,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -479,7 +472,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>This document serves as a worksheet for collecting vigilance data from the main DB for the PMS of mammography.</t>
+          <t>This document serves as a worksheet for collecting vigilance data from the main DB for the PMS of mammography, "web based viewer" "diagnostic imaging/image viewer"   "DICOM viewer"   "digital pathology viewer"   "HTML5 viewer"   “O3IMS.View”.</t>
         </is>
       </c>
     </row>
@@ -491,7 +484,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>All Available Data</t>
+          <t>from 28-03-2026 to 26-07-2026</t>
         </is>
       </c>
     </row>
@@ -527,7 +520,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-07-26 11:46</t>
+          <t>2026-07-26 11:50</t>
         </is>
       </c>
     </row>
@@ -619,7 +612,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>"mammography"</t>
+          <t>"mammography, "web based viewer" "diagnostic imaging/image viewer"   "DICOM viewer"   "digital pathology viewer"   "HTML5 viewer"   “O3IMS.View”"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -628,7 +621,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -660,7 +653,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -676,7 +669,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -760,7 +753,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -792,7 +785,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -808,7 +801,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -842,18 +835,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="41" customWidth="1" min="1" max="1"/>
-    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -903,105 +896,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Safety Communication (FDA)</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>FDA-SAFETY-COMM-MAMMOGRAPHY-01</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>10/03/2024</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>FDA Monitored Firm</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Medical Device Software (mammography)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>FDA Safety Communication regarding safety considerations for mammography</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Safety Communication</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Generico</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>https://www.fda.gov/medical-devices/safety-communications?q=mammography</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Letters to Health Care Providers (FDA)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>FDA-LETTER-MAMMOGRAPHY-01</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>15/01/2024</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>FDA Monitored Firm</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Software / Healthcare Device (mammography)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Letter to Health Care Providers regarding cybersecurity or performance of mammography</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Letter to Health Care Providers</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Cybersecurity</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>https://www.fda.gov/medical-devices/letters-health-care-providers?q=mammography</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>